<commit_message>
Update data processing scripts and figures
Refactored and improved R scripts for data transformation and analysis, including renaming 0_c_main.R to 0_b_main.R, updating data aggregation to handle NA values, and switching parallel processing to sequential. Updated figures, data files, and appendix outputs to reflect latest results and ensure consistency in data handling.
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Joinpoint_APC_results.xlsx
+++ b/Outcome/Appendix/Joinpoint_APC_results.xlsx
@@ -428,7 +428,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>4.77</v>
+        <v>4.78</v>
       </c>
       <c r="D2" t="n">
         <v>2.82</v>
@@ -448,13 +448,13 @@
         <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>-49.88</v>
+        <v>-49.74</v>
       </c>
       <c r="D3" t="n">
-        <v>-65.92</v>
+        <v>-65.83</v>
       </c>
       <c r="E3" t="n">
-        <v>-26.28</v>
+        <v>-26.08</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
@@ -468,13 +468,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>60.65</v>
+        <v>60.62</v>
       </c>
       <c r="D4" t="n">
-        <v>48.56</v>
+        <v>48.53</v>
       </c>
       <c r="E4" t="n">
-        <v>73.72</v>
+        <v>73.69</v>
       </c>
       <c r="F4" t="s">
         <v>8</v>
@@ -488,13 +488,13 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>17.29</v>
+        <v>17.28</v>
       </c>
       <c r="D5" t="n">
-        <v>0.21</v>
+        <v>0.91</v>
       </c>
       <c r="E5" t="n">
-        <v>37.29</v>
+        <v>36.31</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>
@@ -511,7 +511,7 @@
         <v>-15.22</v>
       </c>
       <c r="D6" t="n">
-        <v>-16.9</v>
+        <v>-16.89</v>
       </c>
       <c r="E6" t="n">
         <v>-13.52</v>
@@ -528,13 +528,13 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>40.64</v>
+        <v>40.66</v>
       </c>
       <c r="D7" t="n">
-        <v>31.63</v>
+        <v>31.41</v>
       </c>
       <c r="E7" t="n">
-        <v>50.26</v>
+        <v>50.55</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Refactor age class mapping and improve data processing
Updated AgeClass.csv to use new age groupings and added an Age2 column for more granular mapping. Refactored R scripts to improve age and location-based death data processing, introduced new intermediate variables for clarity, and enhanced reproducibility of ranking calculations. Updated figures, data, and appendix outputs to reflect these changes.
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Joinpoint_APC_results.xlsx
+++ b/Outcome/Appendix/Joinpoint_APC_results.xlsx
@@ -59,7 +59,7 @@
     <t xml:space="preserve">2012/02~2021/03</t>
   </si>
   <si>
-    <t xml:space="preserve">2008/01~2013/10</t>
+    <t xml:space="preserve">2008/01~2013/09</t>
   </si>
   <si>
     <t xml:space="preserve">CFR</t>
@@ -68,10 +68,10 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">2013/11~2016/08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2016/09~2025/12</t>
+    <t xml:space="preserve">2013/10~2016/07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2016/08~2025/12</t>
   </si>
 </sst>
 </file>
@@ -428,13 +428,13 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>4.78</v>
+        <v>4.77</v>
       </c>
       <c r="D2" t="n">
-        <v>2.82</v>
+        <v>3.07</v>
       </c>
       <c r="E2" t="n">
-        <v>6.77</v>
+        <v>6.5</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -448,13 +448,13 @@
         <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>-49.74</v>
+        <v>-50.77</v>
       </c>
       <c r="D3" t="n">
-        <v>-65.83</v>
+        <v>-64.77</v>
       </c>
       <c r="E3" t="n">
-        <v>-26.08</v>
+        <v>-31.19</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
@@ -468,13 +468,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>60.62</v>
+        <v>68.05</v>
       </c>
       <c r="D4" t="n">
-        <v>48.53</v>
+        <v>57.02</v>
       </c>
       <c r="E4" t="n">
-        <v>73.69</v>
+        <v>79.85</v>
       </c>
       <c r="F4" t="s">
         <v>8</v>
@@ -488,13 +488,13 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>17.28</v>
+        <v>17.29</v>
       </c>
       <c r="D5" t="n">
-        <v>0.91</v>
+        <v>1.26</v>
       </c>
       <c r="E5" t="n">
-        <v>36.31</v>
+        <v>35.86</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>
@@ -508,13 +508,13 @@
         <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>-15.22</v>
+        <v>-15.23</v>
       </c>
       <c r="D6" t="n">
-        <v>-16.89</v>
+        <v>-16.86</v>
       </c>
       <c r="E6" t="n">
-        <v>-13.52</v>
+        <v>-13.56</v>
       </c>
       <c r="F6" t="s">
         <v>8</v>
@@ -528,13 +528,13 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>40.66</v>
+        <v>41.8</v>
       </c>
       <c r="D7" t="n">
-        <v>31.41</v>
+        <v>32.68</v>
       </c>
       <c r="E7" t="n">
-        <v>50.55</v>
+        <v>51.55</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -548,13 +548,13 @@
         <v>16</v>
       </c>
       <c r="C8" t="n">
-        <v>-2.65</v>
+        <v>-2.69</v>
       </c>
       <c r="D8" t="n">
-        <v>-7.24</v>
+        <v>-7.29</v>
       </c>
       <c r="E8" t="n">
-        <v>2.17</v>
+        <v>2.15</v>
       </c>
       <c r="F8" t="s">
         <v>17</v>
@@ -568,13 +568,13 @@
         <v>16</v>
       </c>
       <c r="C9" t="n">
-        <v>-40.72</v>
+        <v>-40.17</v>
       </c>
       <c r="D9" t="n">
-        <v>-52.61</v>
+        <v>-52.82</v>
       </c>
       <c r="E9" t="n">
-        <v>-25.83</v>
+        <v>-24.13</v>
       </c>
       <c r="F9" t="s">
         <v>8</v>
@@ -588,13 +588,13 @@
         <v>16</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7</v>
+        <v>-0.15</v>
       </c>
       <c r="D10" t="n">
-        <v>-1.87</v>
+        <v>-2.66</v>
       </c>
       <c r="E10" t="n">
-        <v>3.33</v>
+        <v>2.44</v>
       </c>
       <c r="F10" t="s">
         <v>17</v>

</xml_diff>